<commit_message>
fix(P0-2): correct coordinate-tier calibers per independent review
仅修订定义、分析资格字段、复现说明与断言；不重做 GIS；不改冻结框架。

1) REPRODUCE 口径
- 街道级可归属合计 91 → 283（91 是新增多候选计数，不是街道级总数）
- 门牌级 68 → 门牌粒度可用（含未确认候选）209 = 93 + 116
- 新增「严格点位分析资格」93（95 原始 verified − 2 条兴趣点层级待核）

2) 多候选分母
- 原始 n_candidates>1 = 125，不是 123
- 125 = 91 + 17 + 15 + 2；「123」仅指「多候选且地理编码可用」子集

3) 纠正复核的一处归因
- 复核称 2 条 failed 记录「坐标为空」，实际二者均有坐标：
  P-0bb41fec → 白云区 440111；P-2f0f7abf → 南沙区 440115
  失败原因是落海珠区外（行政区不符）
- 真正无坐标的 failed 是第 3 条 P-45b4cccd（API 错误 30001，无 n_candidates）
- 逐行表新增 geocode返回district / geocode返回adcode 两列使该差异可核验

4) 两条 weak verified
- P-2db0b22d、P-d227f901（level=兴趣点）标「严格点位分析资格=否（待核）」
- **不修改原始 verified=Y，不把 95 降为 93**；95 为状态计数，93 为分析资格

5) 断言
- 新增 G1–G11（含 G3c/G3d 对复核归因的纠正断言）+ 回归 C/A/D
- 合计 25 项全部通过
- 六类互斥合计 340 不变

分类变化：0 条。v1 文件保留不删。
本批为执行方自检，不构成 ChatGPT 独立验收；不宣布 P0 或主报告最终通过。
</commit_message>
<xml_diff>
--- a/03_gis_and_data/p0_reconciliation/P0-3_平安通证据状态表.xlsx
+++ b/03_gis_and_data/p0_reconciliation/P0-3_平安通证据状态表.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3_已取得原件SHA256" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4_待取证清单" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_日期口径对照" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_坐标分层互斥汇总" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_坐标分层互斥汇总_v2" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'S1_金额口径对照'!$A$4:$J$19</definedName>
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'S3_已取得原件SHA256'!$A$4:$F$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'S4_待取证清单'!$A$4:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'S5_日期口径对照'!$A$4:$F$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'S6_坐标分层互斥汇总'!$A$4:$J$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'S6_坐标分层互斥汇总_v2'!$A$4:$J$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2680,25 +2680,25 @@
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>P0-2｜海珠 340 条坐标分层：互斥分类汇总（可由逐行 CSV 复算）</t>
+          <t>P0-2｜海珠 340 条坐标分层：互斥分类汇总 **v2（经独立复核修订）**</t>
         </is>
       </c>
     </row>
     <row r="2" ht="62" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>六类互斥，合计 340。**95 与 116/72 互不相交**；**91 是 116∪72 的子集（68+23）**，不是独立类别。点位级可用仅 95 条；门牌级可用 209 条；街道级可用 283 条。**街道可归属 ≠ 坐标准确**：仅街道级记录不得进入点位/距离/缓冲区/米级结论。</t>
+          <t>六类互斥，合计 340。**93 = 严格点位分析资格**（95 原始verified − 2 条兴趣点层级待核）；**209 = 门牌粒度可用（含 116 条未确认候选）**，不是 209 个已核实服务点；**283 = 街道级可用总数**；**91 = 新增多候选计数**（125 的子集），二者不可混。**街道可归属 ≠ 坐标准确**：仅街道级记录不得进入点位/距离/缓冲区/米级结论。</t>
         </is>
       </c>
     </row>
@@ -2725,27 +2725,27 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
+          <t>其中严格点位分析资格</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>其中门牌粒度可用_含未确认</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>其中街道级可用</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
           <t>其中计入新增91条</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>点位级可用</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>门牌级可用</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>街道级可用</t>
-        </is>
-      </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>可用于点位/距离/缓冲区</t>
+          <t>可用于点位距离缓冲区米级</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -2777,32 +2777,32 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>95</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>93</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>95</t>
-        </is>
-      </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>是（93 条）</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>原始 verified=Y；唯一可用于米级空间运算（其中2条level为弱层级，已单独标注待核）</t>
+          <t>原始verified=Y；其中 2 条层级兴趣点→不具严格点位资格（待核）</t>
         </is>
       </c>
     </row>
@@ -2829,24 +2829,24 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
           <t>68</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>116</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>116</t>
-        </is>
-      </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>geocode 门牌级但未现场确认；可用于街道汇总，点位为候选</t>
+          <t>门牌粒度但未现场确认；可街道汇总，点位为候选</t>
         </is>
       </c>
     </row>
@@ -2881,24 +2881,24 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
           <t>23</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>仅能定街道；坐标可能落街道内任意位置，禁止点位/距离/缓冲区</t>
+          <t>仅能定街道；禁止点位/距离/缓冲区/米级</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>空坐标或失败</t>
+          <t>空坐标或编码失败（3 条 failed：1 条 API 错误、2 条落区外）</t>
         </is>
       </c>
     </row>
@@ -3089,26 +3089,34 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>283</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
           <t>91</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>95</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>209</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>283</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr"/>
-      <c r="J11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>仅 93 条</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>六类互斥。283=街道级可用总数；91=新增多候选计数（125 子集）</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:J11"/>

</xml_diff>

<commit_message>
fix(P0-2): v3 audit hardening per second independent review
仅修正审计问题；不重做 GIS；0 条类别变化；不改冻结框架。

必修1 修复脚本继承缺陷（已证实）
- 01_resolve_coordinates.py 的 except 分支读取上一行 n/lvl/ver
- 实际仅影响 1 条 P-45b4cccd，继承自 P-68e159ad（n=1, level=住宅区）
- 修复：三字段先从当前 r 初始化；API 缺失保持缺失，不写 1
- 重跑明细/分层：仅 2 处字段差异（该条 n_candidates/level → 空），结论层级零变化
- 重算 n_candidates>1 = 125（未硬编码）

必修2 断言修正
- G3c 改为直接检查原始 lng_wgs84/lat_wgs84 非空（不再用 adcode 代替）
- G4 改为从逐行数据分别统计 91/17/15/2 再求和与 125 比较
- 断言输出结构化数组 name/actual/expected/passed；合计 30 项全部通过

必修3 资格分级
- 记录级点位资格 = 93（95 原始 verified − 2 条兴趣点层级待核）
- 最终米级分析资格 = 待坐标系验证（0 条被授权）
- 汇总表不再写「可用于点位距离缓冲区米级=是（93条）」

必修4 标签
- 门牌粒度可用_含未确认候选 → 门牌粒度记录数_含未确认候选（209 = 93 + 116）

必修5 勘误可发现性
- phase2_local_gis/REPRODUCE.md 顶部新增勘误横幅
- 原错误行（91、68）完整保留以便追溯

新增：v3 逐行表/汇总表、geocode审计抽取（340行最小可审计字段）、
v3 断言JSON、v3修订说明、3个v3复现脚本。保留 v1/v2 文件。

本批为执行方自检，不构成 ChatGPT 独立验收；不宣布 P0-2/P0 最终通过。
</commit_message>
<xml_diff>
--- a/03_gis_and_data/p0_reconciliation/P0-3_平安通证据状态表.xlsx
+++ b/03_gis_and_data/p0_reconciliation/P0-3_平安通证据状态表.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3_已取得原件SHA256" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4_待取证清单" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_日期口径对照" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_坐标分层互斥汇总_v2" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_坐标分层互斥汇总_v3" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'S1_金额口径对照'!$A$4:$J$19</definedName>
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'S3_已取得原件SHA256'!$A$4:$F$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'S4_待取证清单'!$A$4:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'S5_日期口径对照'!$A$4:$F$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'S6_坐标分层互斥汇总_v2'!$A$4:$J$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'S6_坐标分层互斥汇总_v3'!$A$4:$J$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2681,10 +2681,10 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -2698,7 +2698,7 @@
     <row r="2" ht="62" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>六类互斥，合计 340。**93 = 严格点位分析资格**（95 原始verified − 2 条兴趣点层级待核）；**209 = 门牌粒度可用（含 116 条未确认候选）**，不是 209 个已核实服务点；**283 = 街道级可用总数**；**91 = 新增多候选计数**（125 的子集），二者不可混。**街道可归属 ≠ 坐标准确**：仅街道级记录不得进入点位/距离/缓冲区/米级结论。</t>
+          <t>六类互斥，合计 340。**93 = 记录级点位资格**（95 原始verified − 2 条兴趣点层级待核）；**最终米级分析资格 = 待坐标系验证**（11区边界坐标系尚未独立验证，93 条不得直接解释为已通过米级/缓冲区分析的最终可用点）；**209 = 门牌粒度可用（含 116 条未确认候选）**，不是 209 个已核实服务点；**283 = 街道级可用总数**；**91 = 新增多候选计数**（125 的子集），二者不可混。**街道可归属 ≠ 坐标准确**：仅街道级记录不得进入点位/距离/缓冲区/米级结论。</t>
         </is>
       </c>
     </row>
@@ -2725,27 +2725,27 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>其中严格点位分析资格</t>
+          <t>其中记录级点位资格</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>其中门牌粒度可用_含未确认</t>
+          <t>最终米级分析资格</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
+          <t>其中门牌粒度记录数_含未确认</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
           <t>其中街道级可用</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>其中计入新增91条</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>可用于点位距离缓冲区米级</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -2782,27 +2782,27 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
+          <t>待坐标系验证</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
           <t>93</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>95</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>是（93 条）</t>
-        </is>
-      </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>原始verified=Y；其中 2 条层级兴趣点→不具严格点位资格（待核）</t>
+          <t>原始verified=Y；2 条层级兴趣点→无记录级点位资格（待核）</t>
         </is>
       </c>
     </row>
@@ -2834,22 +2834,22 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
           <t>116</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>116</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>68</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>否</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -2886,22 +2886,22 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>23</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>否</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -2938,22 +2938,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>否</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -2990,22 +2990,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>否</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -3042,27 +3042,27 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>空坐标或编码失败（3 条 failed：1 条 API 错误、2 条落区外）</t>
+          <t>空坐标或编码失败（3 条 failed：1 条 API 错误无坐标、2 条落区外有坐标）</t>
         </is>
       </c>
     </row>
@@ -3094,27 +3094,27 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
+          <t>待坐标系验证（0 条被授权）</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
           <t>209</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>283</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>91</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>仅 93 条</t>
-        </is>
-      </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>六类互斥。283=街道级可用总数；91=新增多候选计数（125 子集）</t>
+          <t>283=街道级可用总数；91=新增多候选计数（125子集）；93=记录级点位资格，**最终米级分析须待坐标系验证**；209=门牌粒度记录数（93+116），非209个已核实点位</t>
         </is>
       </c>
     </row>

</xml_diff>